<commit_message>
script for Actions class ->seleniumjava
</commit_message>
<xml_diff>
--- a/Excels/Loginpagedata.xlsx
+++ b/Excels/Loginpagedata.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26704"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B06CC6C-0499-4393-852C-B5CD80DCF332}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vvenk\git\FirstMavenautomationproject\Excels\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D38C625-D45B-421B-8707-FC6CE8FDE62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,8 +24,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -28,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>UserName</t>
   </si>
@@ -37,13 +40,22 @@
   </si>
   <si>
     <t>nurse@blueaves.com</t>
+  </si>
+  <si>
+    <t>files@123</t>
+  </si>
+  <si>
+    <t>venkatehdoctor@gmail.com</t>
+  </si>
+  <si>
+    <t>venky@0218</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -399,13 +411,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -413,14 +425,28 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{1D7AC1F0-6215-4A54-BF0D-F58F5516FEF1}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{292048A9-4862-4924-B012-3E4848D82216}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{1B959D33-70F2-40A9-A206-380F6EEE35B4}"/>
+    <hyperlink ref="B3" r:id="rId4" xr:uid="{676A2B36-E397-4508-9789-D8A60D9A2967}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>